<commit_message>
feat(security): implement sprint 2 advanced security hardening (helmet, rate limiting, uploads auth, rh rbac, protheus credentials)
</commit_message>
<xml_diff>
--- a/tests/qa_run/2026-10-17/exports/planejamento_vendas_sem_financeiro.xlsx
+++ b/tests/qa_run/2026-10-17/exports/planejamento_vendas_sem_financeiro.xlsx
@@ -32,7 +32,7 @@
     <t>Gerado em:</t>
   </si>
   <si>
-    <t>17/10/2026, 13:46</t>
+    <t>17/10/2026, 14:01</t>
   </si>
   <si>
     <t>Gerado por:</t>
@@ -491,7 +491,7 @@
     <t>11/12/2026</t>
   </si>
   <si>
-    <t>Documento gerado automaticamente pelo Sistema Lynx  |  17/10/2026, 13:46  |  CONFIDENCIAL — USO INTERNO</t>
+    <t>Documento gerado automaticamente pelo Sistema Lynx  |  17/10/2026, 14:01  |  CONFIDENCIAL — USO INTERNO</t>
   </si>
   <si>
     <t>GUIA DO RELATÓRIO: COMO LER A PLANILHA</t>

</xml_diff>

<commit_message>
feat(optimization): execute backlog - drop 22 orphan tables, purge legacy _arquivo, and implement multi-tenant cron advisory locks
</commit_message>
<xml_diff>
--- a/tests/qa_run/2026-10-17/exports/planejamento_vendas_sem_financeiro.xlsx
+++ b/tests/qa_run/2026-10-17/exports/planejamento_vendas_sem_financeiro.xlsx
@@ -32,7 +32,7 @@
     <t>Gerado em:</t>
   </si>
   <si>
-    <t>17/10/2026, 14:01</t>
+    <t>17/10/2026, 14:09</t>
   </si>
   <si>
     <t>Gerado por:</t>
@@ -491,7 +491,7 @@
     <t>11/12/2026</t>
   </si>
   <si>
-    <t>Documento gerado automaticamente pelo Sistema Lynx  |  17/10/2026, 14:01  |  CONFIDENCIAL — USO INTERNO</t>
+    <t>Documento gerado automaticamente pelo Sistema Lynx  |  17/10/2026, 14:09  |  CONFIDENCIAL — USO INTERNO</t>
   </si>
   <si>
     <t>GUIA DO RELATÓRIO: COMO LER A PLANILHA</t>

</xml_diff>